<commit_message>
cronograma: forro na taxa do material que o nome diz
A fase de Forros punha tudo na taxa de forro de placas de gesso (96109,
1,437 Hh/m²): septo forro/laje, estrutura metálica auxiliar (a área do
forro contada de novo), pintura de forro e o drywall. Nos 27 cronogramas
da base: 6.446 Hh -> ~2.830.

Agora: drywall 96110 1,091 · PVC 96111 0,697 · fibra mineral 104757
0,718 · metálico 97557 0,731 · madeira 96112 2,281 (Hh da nossa base,
insumos em H). Septo/estrutura/pintura saem quando o NOME começa por
eles; tela/arame saem. Forro "tipo a definir" segue na taxa de placas,
como era (decisão do Pedro: sem chute novo).

/exemplo regerado pelo gerador: só a linha de Forros muda (101,7 m²,
14 -> 10 dias). Cronograma já salvo não muda. Mutação 7/7.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/cronograma-exemplo-aiarq.xlsx
+++ b/exemplos/cronograma-exemplo-aiarq.xlsx
@@ -942,11 +942,11 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>2027-01-04</t>
+          <t>2026-12-31</t>
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
@@ -958,11 +958,9 @@
       </c>
       <c r="H15" s="9" t="n"/>
       <c r="I15" s="8" t="n">
-        <v>0.79</v>
-      </c>
-      <c r="J15" s="8" t="n">
-        <v>0.21</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="J15" s="9" t="n"/>
       <c r="K15" s="9" t="n"/>
       <c r="L15" s="9" t="n"/>
     </row>

</xml_diff>